<commit_message>
feat(presupuestos): incorporar escandallo de compra HAM chapa 10eur/m2 omega 6eur/ml a P-2026-0043
</commit_message>
<xml_diff>
--- a/presupuestos/P-2026-0043-rehabilitacion-cubiertas-menorca-dist/presupuesto.xlsx
+++ b/presupuestos/P-2026-0043-rehabilitacion-cubiertas-menorca-dist/presupuesto.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P-2026-0043 Menorca Dist" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Presupuesto Cliente" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Escandallo Costes HAM" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16,10 +17,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="#,##0.00 €"/>
+    <numFmt numFmtId="165" formatCode="0.000"/>
+    <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -66,8 +69,26 @@
       <color rgb="00B91C1C"/>
       <sz val="12"/>
     </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="001E1B4B"/>
+      <sz val="15"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00EF4444"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -96,6 +117,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FEF2F2"/>
         <bgColor rgb="00FEF2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001E1B4B"/>
+        <bgColor rgb="001E1B4B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00ECFDF5"/>
+        <bgColor rgb="00ECFDF5"/>
       </patternFill>
     </fill>
   </fills>
@@ -133,7 +166,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -185,6 +218,37 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="10" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="10" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1076,4 +1140,479 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="25" t="inlineStr">
+        <is>
+          <t>HAM ESTRUCTURAS METÁLICAS - ESTUDIO TÉCNICO INTERNO Y ESCANDALLO DE COMPRA</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="26" t="inlineStr">
+        <is>
+          <t>CONFIDENCIAL: NO ENTREGAR AL CLIENTE · COSTES REALES DE COMPRA Y MÁRGENES</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>PARÁMETROS DE COMPRA DIRECTA HAM:</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Coste compra Chapa Común:</t>
+        </is>
+      </c>
+      <c r="B5" s="22" t="n">
+        <v>10</v>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>€/m²</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Coste compra Omega Galvanizada:</t>
+        </is>
+      </c>
+      <c r="B6" s="22" t="n">
+        <v>6</v>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>€/ml</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Intereje correas nave Alaior:</t>
+        </is>
+      </c>
+      <c r="B7" s="27" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>m (distancia entre correas)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Ratio lineal de omega necesario:</t>
+        </is>
+      </c>
+      <c r="B8" s="28">
+        <f>1/B7</f>
+        <v/>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>ml de omega por m² de faldón</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Mermas y solapes acopio:</t>
+        </is>
+      </c>
+      <c r="B9" s="29" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>5% estándar</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>DESGLOSE DE COSTES DIRECTOS DE EJECUCIÓN (CDT HAM)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="30" t="inlineStr">
+        <is>
+          <t>Capítulo</t>
+        </is>
+      </c>
+      <c r="B12" s="31" t="inlineStr">
+        <is>
+          <t>Concepto de Coste Interno</t>
+        </is>
+      </c>
+      <c r="C12" s="30" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="D12" s="30" t="inlineStr">
+        <is>
+          <t>Medición</t>
+        </is>
+      </c>
+      <c r="E12" s="30" t="inlineStr">
+        <is>
+          <t>Coste Unit. HAM (€)</t>
+        </is>
+      </c>
+      <c r="F12" s="30" t="inlineStr">
+        <is>
+          <t>Coste Total HAM (€)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="17" t="inlineStr">
+        <is>
+          <t>MAT-01</t>
+        </is>
+      </c>
+      <c r="B13" s="18" t="inlineStr">
+        <is>
+          <t>Chapa grecada onda 40 mm / e=0,6 mm prelacada (4.303 m² + 5% solapes/mermas)</t>
+        </is>
+      </c>
+      <c r="C13" s="17" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="D13" s="19" t="n">
+        <v>4518.15</v>
+      </c>
+      <c r="E13" s="20">
+        <f>B5</f>
+        <v/>
+      </c>
+      <c r="F13" s="20">
+        <f>D13*E13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>MAT-02</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>Perfil omega galvanizado Z-275 (4.303 m² x 0,741 ml/m² + 5% solapes longitudinales)</t>
+        </is>
+      </c>
+      <c r="C14" s="17" t="inlineStr">
+        <is>
+          <t>ml</t>
+        </is>
+      </c>
+      <c r="D14" s="19" t="n">
+        <v>3350</v>
+      </c>
+      <c r="E14" s="20">
+        <f>B6</f>
+        <v/>
+      </c>
+      <c r="F14" s="20">
+        <f>D14*E14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="17" t="inlineStr">
+        <is>
+          <t>MAT-03</t>
+        </is>
+      </c>
+      <c r="B15" s="18" t="inlineStr">
+        <is>
+          <t>Tornillería bicromatada a correas + fijación onda alta arandela EPDM + cordón butilo</t>
+        </is>
+      </c>
+      <c r="C15" s="17" t="inlineStr">
+        <is>
+          <t>lote</t>
+        </is>
+      </c>
+      <c r="D15" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" s="20" t="n">
+        <v>7500</v>
+      </c>
+      <c r="F15" s="20">
+        <f>D15*E15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>MAT-04</t>
+        </is>
+      </c>
+      <c r="B16" s="18" t="inlineStr">
+        <is>
+          <t>Placas policarbonato compacto grecado onda 40 mm (126 m² + fijaciones sobreelevadas)</t>
+        </is>
+      </c>
+      <c r="C16" s="17" t="inlineStr">
+        <is>
+          <t>lote</t>
+        </is>
+      </c>
+      <c r="D16" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" s="20" t="n">
+        <v>3978</v>
+      </c>
+      <c r="F16" s="20">
+        <f>D16*E16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="17" t="inlineStr">
+        <is>
+          <t>MAT-05</t>
+        </is>
+      </c>
+      <c r="B17" s="18" t="inlineStr">
+        <is>
+          <t>Rematería plegada 0,60 mm (cumbreras troqueladas, coronaciones, saltos y petos)</t>
+        </is>
+      </c>
+      <c r="C17" s="17" t="inlineStr">
+        <is>
+          <t>lote</t>
+        </is>
+      </c>
+      <c r="D17" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" s="20" t="n">
+        <v>2400</v>
+      </c>
+      <c r="F17" s="20">
+        <f>D17*E17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>MO-01</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>Mano de obra especializada montaje sobrecubierta HAM (cuadrilla oficial ~800 h)</t>
+        </is>
+      </c>
+      <c r="C18" s="17" t="inlineStr">
+        <is>
+          <t>horas</t>
+        </is>
+      </c>
+      <c r="D18" s="19" t="n">
+        <v>800</v>
+      </c>
+      <c r="E18" s="20" t="n">
+        <v>28</v>
+      </c>
+      <c r="F18" s="20">
+        <f>D18*E18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="17" t="inlineStr">
+        <is>
+          <t>LOG-01</t>
+        </is>
+      </c>
+      <c r="B19" s="18" t="inlineStr">
+        <is>
+          <t>Fletes marítimos Península-Menorca + Camión grúa pluma descarga + Alquiler PEMP</t>
+        </is>
+      </c>
+      <c r="C19" s="17" t="inlineStr">
+        <is>
+          <t>lote</t>
+        </is>
+      </c>
+      <c r="D19" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" s="20" t="n">
+        <v>8100</v>
+      </c>
+      <c r="F19" s="20">
+        <f>D19*E19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>PRL-01</t>
+        </is>
+      </c>
+      <c r="B20" s="18" t="inlineStr">
+        <is>
+          <t>Redes anticaídas bajo lucernarios + Líneas de vida temporales + Canon residuos vertedero</t>
+        </is>
+      </c>
+      <c r="C20" s="17" t="inlineStr">
+        <is>
+          <t>lote</t>
+        </is>
+      </c>
+      <c r="D20" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" s="20" t="n">
+        <v>3400</v>
+      </c>
+      <c r="F20" s="20">
+        <f>D20*E20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="E21" s="32" t="inlineStr">
+        <is>
+          <t>COSTE DIRECTO TOTAL (CDT):</t>
+        </is>
+      </c>
+      <c r="F21" s="33">
+        <f>SUM(F13:F20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>CUADRO DE RENTABILIDAD Y BENEFICIO COMERCIAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="34" t="inlineStr">
+        <is>
+          <t>Concepto Económico</t>
+        </is>
+      </c>
+      <c r="B24" s="34" t="inlineStr">
+        <is>
+          <t>Importe (€)</t>
+        </is>
+      </c>
+      <c r="C24" s="34" t="inlineStr">
+        <is>
+          <t>% sobre Venta</t>
+        </is>
+      </c>
+      <c r="D24" s="34" t="inlineStr">
+        <is>
+          <t>Observaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="35" t="inlineStr">
+        <is>
+          <t>Precio de Venta al Cliente (Base Imponible):</t>
+        </is>
+      </c>
+      <c r="B25" s="36">
+        <f>'Presupuesto Cliente'!F27</f>
+        <v/>
+      </c>
+      <c r="C25" s="37" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" s="10" t="inlineStr">
+        <is>
+          <t>PVP ofertado a Menorca Dist</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="35" t="inlineStr">
+        <is>
+          <t>Coste Directo Total de Ejecución HAM:</t>
+        </is>
+      </c>
+      <c r="B26" s="36">
+        <f>F21</f>
+        <v/>
+      </c>
+      <c r="C26" s="37">
+        <f>B26/B25</f>
+        <v/>
+      </c>
+      <c r="D26" s="10" t="inlineStr">
+        <is>
+          <t>Materiales (70%) + MO (20%) + Logística (10%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="38" t="inlineStr">
+        <is>
+          <t>Margen Bruto de Explotación HAM:</t>
+        </is>
+      </c>
+      <c r="B27" s="39">
+        <f>B25-B26</f>
+        <v/>
+      </c>
+      <c r="C27" s="40">
+        <f>B27/B25</f>
+        <v/>
+      </c>
+      <c r="D27" s="41" t="inlineStr">
+        <is>
+          <t>Beneficio neto industrial de la operación</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
fix(presupuestos): ajustar precio de chapa colocada a minimo 55eur/m2 en P-2026-0043
</commit_message>
<xml_diff>
--- a/presupuestos/P-2026-0043-rehabilitacion-cubiertas-menorca-dist/presupuesto.xlsx
+++ b/presupuestos/P-2026-0043-rehabilitacion-cubiertas-menorca-dist/presupuesto.xlsx
@@ -922,7 +922,7 @@
         <v>4303</v>
       </c>
       <c r="E21" s="20" t="n">
-        <v>28.5</v>
+        <v>55</v>
       </c>
       <c r="F21" s="20">
         <f>D21*E21</f>
@@ -949,7 +949,7 @@
         <v>126</v>
       </c>
       <c r="E22" s="20" t="n">
-        <v>54</v>
+        <v>75</v>
       </c>
       <c r="F22" s="20">
         <f>D22*E22</f>
@@ -976,7 +976,7 @@
         <v>1</v>
       </c>
       <c r="E23" s="20" t="n">
-        <v>5850</v>
+        <v>6850</v>
       </c>
       <c r="F23" s="20">
         <f>D23*E23</f>
@@ -1003,7 +1003,7 @@
         <v>1</v>
       </c>
       <c r="E24" s="20" t="n">
-        <v>8600</v>
+        <v>9600</v>
       </c>
       <c r="F24" s="20">
         <f>D24*E24</f>
@@ -1030,7 +1030,7 @@
         <v>1</v>
       </c>
       <c r="E25" s="20" t="n">
-        <v>5400</v>
+        <v>5800</v>
       </c>
       <c r="F25" s="20">
         <f>D25*E25</f>
@@ -1085,7 +1085,7 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>40% a la formalización (72.256,12 € IVA incl.), 30% al inicio del montaje (54.192,09 € IVA incl.) y 30% a la finalización (54.192,09 € IVA incl.)</t>
+          <t>40% a la formalización (129.888,66 € IVA incl.), 30% al inicio del montaje (97.416,50 € IVA incl.) y 30% a la finalización (97.416,49 € IVA incl.)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(presupuestos): actualizar razon social del cliente a Mar Dojan, SL en P-2026-0043
</commit_message>
<xml_diff>
--- a/presupuestos/P-2026-0043-rehabilitacion-cubiertas-menorca-dist/presupuesto.xlsx
+++ b/presupuestos/P-2026-0043-rehabilitacion-cubiertas-menorca-dist/presupuesto.xlsx
@@ -647,7 +647,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Menorca Dist (Distribuciones Menorca)</t>
+          <t>Mar Dojan, SL (Nave Menorca Dist)</t>
         </is>
       </c>
     </row>
@@ -671,7 +671,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>26/10/2026</t>
+          <t>27/10/2026</t>
         </is>
       </c>
     </row>
@@ -1568,7 +1568,7 @@
       </c>
       <c r="D25" s="10" t="inlineStr">
         <is>
-          <t>PVP ofertado a Menorca Dist</t>
+          <t>PVP ofertado a Mar Dojan, SL</t>
         </is>
       </c>
     </row>

</xml_diff>